<commit_message>
added a few new datasets
</commit_message>
<xml_diff>
--- a/1_Data/Sui_2015_unpub/Exp1/Codebook_Sui_2015_unpub_Exp1_Clean.xlsx
+++ b/1_Data/Sui_2015_unpub/Exp1/Codebook_Sui_2015_unpub_Exp1_Clean.xlsx
@@ -744,12 +744,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Accuracy of the participant's response. Coding: 1 = correct (key matches the correct key); 0 = incorrect (key within response keys but wrong); NA = no response; -2 = out-of-range key (key outside the allowed response keys); -3 = early response (before stimulus onset); -4 = late response (after response window)</t>
+          <t>Accuracy of the participant's response. Coding: 1 = correct (key matches the correct key); 0 = incorrect (key within response keys but wrong); 3 = timeout response (probeDur = 1 s, RT &gt;= 1000 ms); 4 = no response (RT = 0)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1 (correct); 0 (incorrect); NA (no response); -2 (out-of-range key); -3 (early response); -4 (late response)</t>
+          <t>1 (correct); 0 (incorrect); 3 (timeout, RT &gt;= 1000 ms); 4 (no response, RT = 0)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">

</xml_diff>